<commit_message>
Fix workbook that Excel refused to open
Each formula cell carried two <v> elements. openpyxl writes an empty <v/> after
the <f>, and the cached-value injection appended a second one instead of
replacing it. CT_Cell allows at most one <v>, so openpyxl and LibreOffice read
the file while Excel rejected it.

The injection now substitutes the existing <v/> and asserts that every formula
cell was patched. It also sets fullCalcOnLoad on the workbook so Excel
recalculates on open and the cached values can never drift from the formulas.

Also adds the glossary sheet builder, which was missing from the script set, so
the workbook is reproducible end to end.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QmVe5dRye8Na5NC4UqHqFY
</commit_message>
<xml_diff>
--- a/outputs/solfacil/Solfacil_Securitizacoes_Comparativo.xlsx
+++ b/outputs/solfacil/Solfacil_Securitizacoes_Comparativo.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="FIDC" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="CRI" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Como ler" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FIDC" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRI" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Como ler" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -2565,37 +2565,30 @@
       <c r="B55" s="8">
         <f>SUM(B52:B54)</f>
         <v>83.7</v>
-        <v/>
       </c>
       <c r="C55" s="8">
         <f>SUM(C52:C54)</f>
         <v>94.0</v>
-        <v/>
       </c>
       <c r="D55" s="8">
         <f>SUM(D52:D54)</f>
         <v>17.5</v>
-        <v/>
       </c>
       <c r="E55" s="8">
         <f>SUM(E52:E54)</f>
         <v>67.5</v>
-        <v/>
       </c>
       <c r="F55" s="8">
         <f>SUM(F52:F54)</f>
         <v>141.1</v>
-        <v/>
       </c>
       <c r="G55" s="8">
         <f>SUM(G52:G54)</f>
         <v>211.0</v>
-        <v/>
       </c>
       <c r="H55" s="8">
         <f>SUM(H52:H54)</f>
         <v>619.7</v>
-        <v/>
       </c>
     </row>
     <row r="56">
@@ -2607,37 +2600,30 @@
       <c r="B56" s="9">
         <f>IF(B55=0,0,B52/B55)</f>
         <v>0.6356033453</v>
-        <v/>
       </c>
       <c r="C56" s="9">
         <f>IF(C55=0,0,C52/C55)</f>
         <v>0.7287234043</v>
-        <v/>
       </c>
       <c r="D56" s="9">
         <f>IF(D55=0,0,D52/D55)</f>
         <v>1.0</v>
-        <v/>
       </c>
       <c r="E56" s="9">
         <f>IF(E55=0,0,E52/E55)</f>
         <v>0.7911111111</v>
-        <v/>
       </c>
       <c r="F56" s="9">
         <f>IF(F55=0,0,F52/F55)</f>
         <v>0.6683203402</v>
-        <v/>
       </c>
       <c r="G56" s="9">
         <f>IF(G55=0,0,G52/G55)</f>
         <v>0.6639810427</v>
-        <v/>
       </c>
       <c r="H56" s="9">
         <f>IF(H55=0,0,H52/H55)</f>
         <v>0.7398741326</v>
-        <v/>
       </c>
     </row>
     <row r="57">
@@ -2649,37 +2635,30 @@
       <c r="B57" s="9">
         <f>IF(B55=0,0,B53/B55)</f>
         <v>0.3249701314</v>
-        <v/>
       </c>
       <c r="C57" s="9">
         <f>IF(C55=0,0,C53/C55)</f>
         <v>0.1489361702</v>
-        <v/>
       </c>
       <c r="D57" s="9">
         <f>IF(D55=0,0,D53/D55)</f>
         <v>0.0</v>
-        <v/>
       </c>
       <c r="E57" s="9">
         <f>IF(E55=0,0,E53/E55)</f>
         <v>0.1348148148</v>
-        <v/>
       </c>
       <c r="F57" s="9">
         <f>IF(F55=0,0,F53/F55)</f>
         <v>0.2097802977</v>
-        <v/>
       </c>
       <c r="G57" s="9">
         <f>IF(G55=0,0,G53/G55)</f>
         <v>0.1867298578</v>
-        <v/>
       </c>
       <c r="H57" s="9">
         <f>IF(H55=0,0,H53/H55)</f>
         <v>0.2078425044</v>
-        <v/>
       </c>
     </row>
     <row r="58">
@@ -2691,37 +2670,30 @@
       <c r="B58" s="9">
         <f>IF(B55=0,0,B54/B55)</f>
         <v>0.0394265233</v>
-        <v/>
       </c>
       <c r="C58" s="9">
         <f>IF(C55=0,0,C54/C55)</f>
         <v>0.1223404255</v>
-        <v/>
       </c>
       <c r="D58" s="9">
         <f>IF(D55=0,0,D54/D55)</f>
         <v>0.0</v>
-        <v/>
       </c>
       <c r="E58" s="9">
         <f>IF(E55=0,0,E54/E55)</f>
         <v>0.0740740741</v>
-        <v/>
       </c>
       <c r="F58" s="9">
         <f>IF(F55=0,0,F54/F55)</f>
         <v>0.1218993622</v>
-        <v/>
       </c>
       <c r="G58" s="9">
         <f>IF(G55=0,0,G54/G55)</f>
         <v>0.1492890995</v>
-        <v/>
       </c>
       <c r="H58" s="9">
         <f>IF(H55=0,0,H54/H55)</f>
         <v>0.0522833629</v>
-        <v/>
       </c>
     </row>
     <row r="59">
@@ -2733,37 +2705,30 @@
       <c r="B59" s="10">
         <f>IF(B55=0,0,(B53+B54)/B55)</f>
         <v>0.3643966547</v>
-        <v/>
       </c>
       <c r="C59" s="10">
         <f>IF(C55=0,0,(C53+C54)/C55)</f>
         <v>0.2712765957</v>
-        <v/>
       </c>
       <c r="D59" s="10">
         <f>IF(D55=0,0,(D53+D54)/D55)</f>
         <v>0.0</v>
-        <v/>
       </c>
       <c r="E59" s="10">
         <f>IF(E55=0,0,(E53+E54)/E55)</f>
         <v>0.2088888889</v>
-        <v/>
       </c>
       <c r="F59" s="10">
         <f>IF(F55=0,0,(F53+F54)/F55)</f>
         <v>0.3316796598</v>
-        <v/>
       </c>
       <c r="G59" s="10">
         <f>IF(G55=0,0,(G53+G54)/G55)</f>
         <v>0.3360189573</v>
-        <v/>
       </c>
       <c r="H59" s="10">
         <f>IF(H55=0,0,(H53+H54)/H55)</f>
         <v>0.2601258674</v>
-        <v/>
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
@@ -3268,12 +3233,10 @@
       <c r="B28" s="16">
         <f>SUM(B22:B27)</f>
         <v>470.599</v>
-        <v/>
       </c>
       <c r="C28" s="16">
         <f>SUM(C22:C27)</f>
         <v>627.647</v>
-        <v/>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">

</xml_diff>